<commit_message>
Doc: Ajustes na tabela de regras de negócio e história de usuário
</commit_message>
<xml_diff>
--- a/Arquivos-Escopo/RegrasDeNegocio 1.xlsx
+++ b/Arquivos-Escopo/RegrasDeNegocio 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\AgroFlux2026\Arquivos-Escopo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\OneDrive - SESISENAISP - Escolas\Área de Trabalho\AgroFlux2026\Arquivos-Escopo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7CD2128-706C-40DC-AEEA-DA3EE2374DF8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{D7CD2128-706C-40DC-AEEA-DA3EE2374DF8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{54335625-8650-4289-89F9-9B17E4F9629D}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>REGRAS DE NEGÓCIO</t>
   </si>
@@ -92,13 +92,23 @@
     <t xml:space="preserve">  O USUÁRIO SÓ PODE ACESSAR O SISTEMA SE ESTIVER AUTENTICADO</t>
   </si>
   <si>
-    <t>DADOS JA EXISTENTE</t>
-  </si>
-  <si>
     <t>ATUALIZAÇAO DE ESTOQUE</t>
   </si>
   <si>
     <t>ALERTA DE ESTOQUE BAIXO</t>
+  </si>
+  <si>
+    <t>DADOS JÁ EXISTENTE</t>
+  </si>
+  <si>
+    <t>EXCLUSÃO DE PRODUTOS</t>
+  </si>
+  <si>
+    <t>CADASTRO OU EDIÇÃO DE 
+USUÁRIO</t>
+  </si>
+  <si>
+    <t>CPF USUÁRIO</t>
   </si>
 </sst>
 </file>
@@ -184,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -194,9 +204,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -410,11 +417,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -431,7 +438,7 @@
       <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -443,9 +450,9 @@
         <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>17</v>
       </c>
     </row>
@@ -454,9 +461,9 @@
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>12</v>
       </c>
     </row>
@@ -465,9 +472,9 @@
         <v>8</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -475,8 +482,10 @@
       <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="6" t="s">
+      <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -484,8 +493,10 @@
       <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="6" t="s">
+      <c r="C9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>15</v>
       </c>
     </row>
@@ -493,8 +504,10 @@
       <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="6" t="s">
+      <c r="C10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Doc: Correção da RN002
</commit_message>
<xml_diff>
--- a/Arquivos-Escopo/RegrasDeNegocio 1.xlsx
+++ b/Arquivos-Escopo/RegrasDeNegocio 1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\OneDrive - SESISENAISP - Escolas\Área de Trabalho\AgroFlux2026\Arquivos-Escopo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\AgroFlux2026\Arquivos-Escopo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{D7CD2128-706C-40DC-AEEA-DA3EE2374DF8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{54335625-8650-4289-89F9-9B17E4F9629D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BEA6F09-87DE-4DBF-A62D-23D223CA3EAA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,10 +85,6 @@
  POSSUIR CPF VÁLIDO E ÚNICO</t>
   </si>
   <si>
-    <t xml:space="preserve">     DADOS DUPLICADOS NÃO
-       PODEM SER CADASTRADOS</t>
-  </si>
-  <si>
     <t xml:space="preserve">  O USUÁRIO SÓ PODE ACESSAR O SISTEMA SE ESTIVER AUTENTICADO</t>
   </si>
   <si>
@@ -109,6 +105,10 @@
   </si>
   <si>
     <t>CPF USUÁRIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     DADOS DUPLICADOS NÃO
+       PODEM SER CADASTRADOS(COMO POR EXEMPLO PODUTOS QUE JÁ FORAM ANTES CADASTRADOS, OU NO CASO DE FÚNCIONARIOS, EMAIL QUE JÁ ESTEJA SENDO UTILIZADO)</t>
   </si>
 </sst>
 </file>
@@ -442,18 +442,18 @@
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" ht="47.4" customHeight="1" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="151.19999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -461,7 +461,7 @@
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>12</v>
@@ -472,7 +472,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>13</v>
@@ -483,7 +483,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>14</v>
@@ -494,7 +494,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>15</v>
@@ -505,7 +505,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>16</v>

</xml_diff>